<commit_message>
feat: latest content sync
</commit_message>
<xml_diff>
--- a/static/demo/downloads/gap-analysis.xlsx
+++ b/static/demo/downloads/gap-analysis.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap Analysis" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,8 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="4">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,28 +29,41 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="001B2A4A"/>
       <sz val="14"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00333333"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00333333"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -57,8 +73,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F5F5F5"/>
-        <bgColor rgb="00F5F5F5"/>
+        <fgColor rgb="00FAFAFA"/>
+        <bgColor rgb="00FAFAFA"/>
       </patternFill>
     </fill>
   </fills>
@@ -88,22 +104,90 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00B85042"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFEBEE"/>
+          <bgColor rgb="00FFEBEE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00D4A843"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF8E1"/>
+          <bgColor rgb="00FFF8E1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="002C5F2D"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E8F5E9"/>
+          <bgColor rgb="00E8F5E9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -466,239 +550,525 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="35" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AI Maturity Gap Analysis — Meridian Healthcare</t>
+          <t>Gap Analysis: Current State vs Target State</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Dimension</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Gap</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Investment Required</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Recommended Action</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Recommendation</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Timeline</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Investment</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Expected Impact</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Owner</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Data Governance</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D3" s="5">
+        <f>C3-B3</f>
+        <v/>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>$450K</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Deploy governance framework with 6 data stewards</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Hire AI/ML Lead + 2 ML Engineers</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Month 1-2</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>$420K/yr</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>Unblock NLP pilot</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>CTO</t>
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Data Architecture</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C4" s="9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D4" s="9">
+        <f>C4-B4</f>
+        <v/>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>$380K</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr">
+        <is>
+          <t>Implement MDM platform and API-based integration layer</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Analytics Capability</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D5" s="5">
+        <f>C5-B5</f>
+        <v/>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>$250K</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>Expand self-service analytics and hire 2 data scientists</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>AI/ML Operations</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D6" s="9">
+        <f>C6-B6</f>
+        <v/>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F6" s="10" t="inlineStr">
+        <is>
+          <t>$620K</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>Build MLOps pipeline with CI/CD and model monitoring</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Data Culture</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Deploy AI governance framework</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Month 1-3</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>$280K</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>HIPAA + EU AI Act readiness</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>CDO</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Implement MLflow for model management</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Month 2-4</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>$85K</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>NLP pilot to production in 6 weeks</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>AI/ML Lead</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Establish data quality program</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Month 3-6</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>$150K</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>Data quality 62% → 85%</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Head of Gov</t>
+      <c r="C7" s="5" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D7" s="5">
+        <f>C7-B7</f>
+        <v/>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>$180K</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Launch data literacy program targeting 500 employees</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Create dedicated AI budget line</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Month 1</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>$0</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>Visibility and accountability</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>CFO</t>
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Data Quality</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D8" s="9">
+        <f>C8-B8</f>
+        <v/>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>$320K</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>Deploy automated quality monitoring across 12 data domains</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Build use case pipeline process</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Month 2-4</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>$60K</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>Systematic AI opportunity capture</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>Use Case Lead</t>
-        </is>
-      </c>
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>TOTAL INVESTMENT</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr"/>
+      <c r="C9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>$2,200K</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="D3:D8">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
+      <formula>1.5</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="between" dxfId="1">
+      <formula>0.8</formula>
+      <formula>1.5</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="lessThan" dxfId="2">
+      <formula>0.8</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E3:E8">
+    <cfRule type="expression" priority="4" dxfId="0">
+      <formula>E3="Critical"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="5" dxfId="1">
+      <formula>E3="High"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002D4A7A"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="35" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Implementation Timeline</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Initiative</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Q2 2026</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Q3 2026</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Q1 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Governance framework</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>Operationalize</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>Optimize</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>MDM platform</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Vendor select</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>Implement</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Migrate data</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Go-live</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>MLOps pipeline</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Data quality monitoring</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>Requirements</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>Expand</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>Full coverage</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Data literacy program</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Curriculum</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Pilot (50)</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Scale (200)</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>Scale (500)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Self-service analytics</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Tool evaluation</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>Deploy</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>Training</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>Adoption push</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>